<commit_message>
Updated RIOT Logic spreadsheet
</commit_message>
<xml_diff>
--- a/riot_logic.xlsx
+++ b/riot_logic.xlsx
@@ -1033,23 +1033,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="F12:F13"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="D16:D17"/>
-    <mergeCell ref="E12:E15"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="A20:A36"/>
-    <mergeCell ref="C11:C17"/>
-    <mergeCell ref="D11:D15"/>
-    <mergeCell ref="A1:A17"/>
-    <mergeCell ref="B1:B2"/>
-    <mergeCell ref="B3:B17"/>
-    <mergeCell ref="C3:C10"/>
-    <mergeCell ref="D3:D6"/>
-    <mergeCell ref="D7:D10"/>
     <mergeCell ref="F24:F25"/>
     <mergeCell ref="F22:F23"/>
     <mergeCell ref="B35:B36"/>
@@ -1065,6 +1048,23 @@
     <mergeCell ref="E33:E34"/>
     <mergeCell ref="E22:E25"/>
     <mergeCell ref="E27:E28"/>
+    <mergeCell ref="A20:A36"/>
+    <mergeCell ref="C11:C17"/>
+    <mergeCell ref="D11:D15"/>
+    <mergeCell ref="A1:A17"/>
+    <mergeCell ref="B1:B2"/>
+    <mergeCell ref="B3:B17"/>
+    <mergeCell ref="C3:C10"/>
+    <mergeCell ref="D3:D6"/>
+    <mergeCell ref="D7:D10"/>
+    <mergeCell ref="F12:F13"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="E12:E15"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="E9:E10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>